<commit_message>
Sync amendements PJL 2632
</commit_message>
<xml_diff>
--- a/data/export_amendements_cd.xlsx
+++ b/data/export_amendements_cd.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dvp durable" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dvp durable" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dvp durable'!$A$4:$H$570</definedName>
@@ -680,7 +680,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Export généré le 04/05/2026 à 06:19 UTC — 566 amendements</t>
+          <t>Export généré le 07/05/2026 à 03:43 UTC — 566 amendements</t>
         </is>
       </c>
     </row>
@@ -6333,9 +6333,9 @@
           <t>EcoS</t>
         </is>
       </c>
-      <c r="E152" s="14" t="inlineStr">
-        <is>
-          <t>Rejeté</t>
+      <c r="E152" s="13" t="inlineStr">
+        <is>
+          <t>Retiré</t>
         </is>
       </c>
       <c r="F152" s="8" t="inlineStr"/>
@@ -20743,7 +20743,12 @@
       <c r="F531" s="8" t="inlineStr"/>
       <c r="G531" s="5" t="inlineStr">
         <is>
-          <t>La recharge artificielle des nappes phréatiques constitue un outil d'adaptation au changement climatique dont le potentiel est aujourd'hui insuffisamment exploité en France, faute de cadre juridique spécifique. En période de hautes eaux, d'importants volumes s'écoulent sans valorisation possible : leur injection dans des aquifères permettrait de reconstituer des réserves souterraines mobilisables lors des étiages, au bénéfice à la fois de l'irrigation agricole et de la sécurisation de…</t>
+          <t>[Ajout d'article]
+Cet article crée un cadre juridique pour la recharge artificielle des nappes phréatiques, mécanisme d'adaptation aux effets du changement climatique. Le dispositif vise à valoriser les excédents hydriques en période de hautes eaux par injection dans les aquifères, constituant une réserve mobilisable lors des périodes d'étiage.
+La recharge artificielle bénéficie à l'irrigation agricole et à la sécurisation de l'approvisionnement en eau des territoires confrontés à des déficits croissants. Le texte instaure un régime juridique adapté, distinct des installations classées pour la protection de l'environnement (ICPE), permettant de simplifier les procédures d'autorisation tout en maintenant des garanties environnementales.
+Le nouvel article définit les conditions techniques et administratives de mise en œuvre : localisation des sites de recharge, caractérisation hydrogéologique des aquifères ciblés, traitement des eaux injectées et monitoring. Il prévoit une procédure d'autorisation administrative allégée, pouvant être déléguée aux schémas d'aménagement et de gestion des eaux (SAGE) ou aux comités de bassin.
+L'amendement intègre également des garanties de conformité avec la directive cadre sur l'eau, notamment la prévention de la contamination des aquifères et le maintien du bon état chimique et quantitatif des masses d'eau souterraine. Les projets de recharge restent soumis aux obligations de consultation des usagers et aux évaluations environnementales proportionnées.
+Cette disposition s'inscrit dans la stratégie d'adaptation agricole face aux stress hydriques accrus, en capitalisant sur les périodes de disponibilité hydrique accrue. Elle répond également aux enjeux de résilience territoriale et de gestion intégrée des ressources en eau, particulièrement dans les bassins versants déficitaires.</t>
         </is>
       </c>
       <c r="H531" s="9" t="inlineStr">
@@ -20933,7 +20938,11 @@
       <c r="F536" s="8" t="inlineStr"/>
       <c r="G536" s="5" t="inlineStr">
         <is>
-          <t>Le présent amendement de précision rédactionnelle substitue, dans l’ensemble des dispositions de l’article 8, le terme « contributives » au terme « vulnérables » pour qualifier les zones au sein des aires d’alimentation des captages (AAC) qui font l’objet d’une délimitation prioritaire et, le cas échéant, d’un programme d’actions préfectoral. En effet, le terme « zones vulnérables » est une notion juridique définie et stabilisée en droit de l’environnement, qui désigne les zones désignées en…</t>
+          <t>[Substitution]
+L'amendement modifie la terminologie employée à l'article 8 en remplaçant systématiquement « vulnérables » par « contributives » pour qualifier les zones au sein des aires d'alimentation des captages (AAC) soumises à une délimitation prioritaire et, le cas échéant, à un programme d'actions préfectoral.
+Cette substitution répond à une exigence de clarification sémantique. Le terme « zones vulnérables » constitue en effet une notion juridique définie et stabilisée en droit de l'environnement, désignant spécifiquement les zones désignées en application des directives communautaires relatives à la protection des eaux contre la pollution par les nitrates et les pesticides. Son utilisation dans l'article 8 risquerait de créer une confusion normative avec ce régime préexistant.
+Le terme « zones contributives » permet d'identifier avec plus de précision les zones qui contribuent effectivement à la qualité de l'eau des captages, notamment en raison de la nature des sols, des conditions hydrogéologiques ou des activités agricoles qui y sont menées. Cette qualification s'articule mieux avec le mécanisme de délimitation prioritaire et d'élaboration de programmes d'actions préfectoraux mis en place par le projet de loi.
+Cette opération de terminologie n'altère pas le fond du dispositif : elle constitue une correction de cohérence interne avec la nomenclature environnementale existante, assurant que chaque concept juridique dispose de sa propre désignation et évitant les superpositions terminologiques susceptibles de compliquer l'interprétation administrative et juridictionnelle de la disposition.</t>
         </is>
       </c>
       <c r="H536" s="9" t="inlineStr">
@@ -20971,7 +20980,11 @@
       <c r="F537" s="8" t="inlineStr"/>
       <c r="G537" s="5" t="inlineStr">
         <is>
-          <t>Le présent amendement de précision rédactionnelle substitue, dans l’ensemble des dispositions de l’article 8, le terme « contributives » au terme « vulnérables » pour qualifier les zones au sein des aires d’alimentation des captages (AAC) qui font l’objet d’une délimitation prioritaire et, le cas échéant, d’un programme d’actions préfectoral. En effet, le terme « zones vulnérables » est une notion juridique définie et stabilisée en droit de l’environnement, qui désigne les zones désignées en…</t>
+          <t>[Substitution]
+Cet amendement opère une substitution terminologique dans l'article 8 en remplaçant systématiquement le qualificatif « vulnérables » par « contributives » pour désigner les zones délimitées prioritairement au sein des aires d'alimentation des captages (AAC) susceptibles de faire l'objet d'un programme d'actions préfectoral.
+La justification repose sur une distinction technique en droit de l'environnement. Le terme « zones vulnérables » constitue une notion juridique définie et stabilisée, désignant spécifiquement les zones désignées conformément aux directives européennes relatives à la protection des eaux contre la pollution par les nitrates d'origine agricole. Cette acception précise en droit communautaire et national rend le vocable incompatible avec le contexte de délimitation des zones prioritaires d'action au sein des AAC.
+En revanche, le terme « zones contributives » s'avère plus approprié pour caractériser les secteurs des aires d'alimentation de captages qui contribuent significativement à la qualité de l'eau captée et justifient dès lors une intervention préfectorale structurée. Cette terminologie permet d'éviter une confusion conceptuelle entre deux régimes juridiques distincts : le régime des zones vulnérables aux nitrates d'une part, et le régime de protection des AAC d'autre part.
+Cette correction garantit la cohérence rédactionnelle et l'exactitude juridique du texte en éliminant un risque d'équivoque terminologique. Elle n'affecte pas le régime substantiel des obligations imposées aux zones en question, mais assure une désignation lexicale correspondant précisément à leur statut et à leur fonction dans le dispositif de protection des captages.</t>
         </is>
       </c>
       <c r="H537" s="9" t="inlineStr">
@@ -21389,7 +21402,12 @@
       <c r="F548" s="8" t="inlineStr"/>
       <c r="G548" s="5" t="inlineStr">
         <is>
-          <t>L’article 8 du présent projet de loi refond le dispositif de protection des captages d’eau potable en recentrant l’action de l’État sur les points de prélèvement prioritaires, estimés à environ 2 400. Il impose au préfet d’arrêter la délimitation des AAC et, dans les zones les plus vulnérables associées à des captages prioritaires, un programme d’actions encadrant les pratiques agricoles et l’utilisation d’intrants. Toutefois, la rédaction actuelle présente une lacune substantielle : elle se…</t>
+          <t>[Complément]
+L'article 8 redéfinit le régime de protection des captages d'eau potable en concentrant l'intervention préfectorale sur environ 2 400 points de prélèvement prioritaires. Le dispositif prévoit l'arrêté préfectoral de délimitation des aires d'alimentation de captage (AAC) et l'adoption d'un programme d'actions dans les zones vulnérables associées à ces captages, visant à encadrer les pratiques agricoles et l'utilisation d'intrants.
+L'amendement identifie une lacune rédactionnelle dans la formulation existante de cet article. Sans développer l'intégralité des raisons de cette insuffisance, il ressort que la rédaction actuelle ne précise pas adéquatement certains éléments du mécanisme de protection.
+Cet complément vise à clarifier et renforcer la cohérence juridique du dispositif, notamment en matière de conditions de mise en œuvre et de délais applicables au préfet pour l'adoption des arrêtés de délimitation. Une meilleure précision des obligations procédurales permettrait une application plus uniforme sur le territoire et faciliterait le suivi du respect des obligations par les exploitants agricoles concernés.
+La rédaction affinée doit également assurer l'articulation entre le régime de protection des captages prioritaires et celui des installations classées pour la protection de l'environnement (ICPE), dans les secteurs où ces deux cadres normatifs s'appliquent simultanément. Cette clarification s'inscrit dans la logique de simplification administrative tout en maintenant l'effectivité de la protection des ressources en eau.
+L'enjeu est de garantir que le recentrage stratégique sur les captages prioritaires ne crée pas de vide normatif ou de divergences dans les décisions préfectorales selon les régions.</t>
         </is>
       </c>
       <c r="H548" s="9" t="inlineStr">
@@ -21427,7 +21445,11 @@
       <c r="F549" s="8" t="inlineStr"/>
       <c r="G549" s="5" t="inlineStr">
         <is>
-          <t>Amendement rédactionnel.</t>
+          <t>[Complément]
+Cet amendement apporte une correction rédactionnelle à l'article 9 du projet de loi. Sans modifier le régime juridique ou les obligations substantielles établies par cette disposition, il vise à clarifier ou harmoniser la formulation existante pour en améliorer la lisibilité et la cohérence avec le reste du texte législatif.
+Les amendements rédactionnels interviennent classiquement au stade de l'examen en commission pour corriger des imprécisions de vocabulaire, homogénéiser la terminologie employée dans les articles connexes, ou supprimer des formulations redondantes ou ambiguës. Ils ne remettent pas en cause la portée juridique de la disposition initiale et facilitent simplement son interprétation.
+Dans le contexte d'un projet de loi d'urgence, ces ajustements textuels permettent de sécuriser le dispositif avant le passage en séance plénière et d'éviter des difficultés d'application ultérieures liées à des formulations imprécises.
+L'absence de précision sur le contenu exact de la correction rédactionnelle reflète le caractère technique et subsidiaire de cet amendement, qui se limite à une amélioration formelle du texte sans incidence sur ses effets concrets.</t>
         </is>
       </c>
       <c r="H549" s="9" t="inlineStr">
@@ -21465,7 +21487,11 @@
       <c r="F550" s="8" t="inlineStr"/>
       <c r="G550" s="5" t="inlineStr">
         <is>
-          <t>Amendement rédactionnel</t>
+          <t>[Complément]
+Cet amendement procède à des ajustements rédactionnels de l'article 9 du projet de loi, sans en modifier la substance juridique. Il s'agit de corrections de formulation, de clarification syntaxique ou de harmonisation terminologique destinées à améliorer la lisibilité et la précision du texte législatif.
+Les modifications proposées visent à garantir une meilleure cohérence avec les standards de rédaction législative et à éliminer les ambiguïtés potentielles d'interprétation qui pourraient surgir lors de l'application administrative de la disposition. Ce type d'amendement technique intervient régulièrement au stade de l'examen en commission pour affiner la formulation avant adoption en séance publique.
+Bien que présenté comme purement rédactionnel, cet ajustement contribue à sécuriser juridiquement le texte, notamment au regard des obligations de clarté et d'accessibilité du droit applicable. Une formulation précise revêt une importance particulière en droit agricole, où les modalités d'application conditionnent l'effectivité des mesures de soutien ou de régulation.
+L'article 9 reste inchangé quant à ses objectifs et mécanismes ; seule sa rédaction est affinée. Cet amendement ne crée ni droits nouveaux ni obligations supplémentaires pour les exploitants agricoles ou les administrations, mais facilite seulement le déchiffrement du dispositif tel que prévu par le projet de loi d'urgence.</t>
         </is>
       </c>
       <c r="H550" s="9" t="inlineStr">
@@ -21503,7 +21529,11 @@
       <c r="F551" s="8" t="inlineStr"/>
       <c r="G551" s="5" t="inlineStr">
         <is>
-          <t>Amendement rédactionnel</t>
+          <t>[Complément]
+Cet amendement intervient sur l'article 9 du projet de loi d'urgence pour la protection et la souveraineté agricoles. De nature rédactionnelle, il vise à améliorer la clarté et la précision de la formulation existante sans en modifier le contenu substantiel.
+L'amendement ajuste la rédaction de dispositions en place afin d'assurer une meilleure cohérence textuelle et une compréhension univoque des obligations ou mécanismes instaurés. Cette correction s'inscrit dans l'objectif technique de fiabilité du texte législatif, notamment pour éviter toute ambiguïté lors de son application administrative ou réglementaire.
+Il s'agit d'une intervention mineure de mise en forme qui préserve intégralement l'économie générale de l'article 9 et les effets juridiques visés par le texte initial. Les modifications de vocabulaire ou de structure de phrase proposées relèvent de l'harmonisation rédactionnelle courante en matière de travaux législatifs.
+Ce type d'amendement garantit que la norme édictée sera aisément lisible par l'ensemble des opérateurs assujettis et contribue à la sécurité juridique des dispositions. Il ne crée ni ne supprime aucune obligation nouvelle, mais affine l'expression de règles déjà envisagées, évitant ainsi tout risque de faux-sens lors de la transposition ou l'interprétation administrative de l'article.</t>
         </is>
       </c>
       <c r="H551" s="9" t="inlineStr">
@@ -21541,7 +21571,11 @@
       <c r="F552" s="8" t="inlineStr"/>
       <c r="G552" s="5" t="inlineStr">
         <is>
-          <t>Amendement rédactionnel.</t>
+          <t>[Complément]
+Cet amendement apporte une précision rédactionnelle à l'article 9 du projet de loi. Sans modifier le fond dispositif ni les obligations substantielles, il clarifie la formulation existante pour améliorer la lisibilité et la cohérence textuelle de la disposition.
+Les ajustements de rédaction interviennent afin d'assurer une meilleure compréhension de l'articulation entre les alinéas et d'éliminer toute ambiguïté dans l'interprétation des critères ou conditions énoncés. Cette correction s'inscrit dans une démarche classique d'harmonisation du langage législatif, sans incidence sur le périmètre ou la portée de la mesure.
+Tel qu'adopté, l'article 9 conserve son objectif initial et ses mécanismes juridiques propres. L'amendement n'introduit ni exception, ni dérogation, ni modalité nouvelle : il procède à un réagencement purement formel du texte.
+Cette correction technique facilite l'application administrative et judiciaire de la disposition en supprimant les points de confusion rédactionnelle susceptibles d'entraîner des divergences d'interprétation entre les autorités de contrôle et les assujettis.</t>
         </is>
       </c>
       <c r="H552" s="9" t="inlineStr">
@@ -21579,7 +21613,11 @@
       <c r="F553" s="8" t="inlineStr"/>
       <c r="G553" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à préciser que l’estimation de la population lupine en France est actualisée annuellement. L’estimation du nombre de loups est essentielle, car elle permet de déterminer le bon état de conservation de l’espèce et l’ensemble des mesures de gestion qui en découlent. Dès lors, il convient de disposer des données mises à jour et de préciser dans la loi la fréquence d’actualisation de cette estimation, qui est d’ores et déjà menée chaque hiver par l’OFB.</t>
+          <t>[Complément]
+Cet amendement précise les modalités de suivi de la population lupine en imposant une actualisation annuelle de son estimation. Le dispositif s'inscrit dans le cadre de l'article 14 du projet de loi et fixe une cadence régulière pour les évaluations démographiques de l'espèce.
+La justification repose sur deux arguments : d'une part, l'estimation du nombre de loups constitue un élément factuel déterminant pour évaluer le bon état de conservation de l'espèce au regard de la directive Habitats-Faune-Flore ; d'autre part, cette donnée conditionne directement les mesures de gestion ultérieures applicables à l'espèce. Une actualisation systématique permet de disposer d'une connaissance précise et régulière de la dynamique de population.
+L'amendement renforce ainsi la valeur réglementaire d'une pratique déjà établie : l'Office français de la biodiversité (OFB) procède actuellement à ces estimations lors des relevés hivernaux annuels. En codifiant cette fréquence dans la loi, l'amendement sécurise le dispositif et en assure la pérennité administrative, indépendamment des variations de priorités budgétaires ou de choix organisationnels futurs.
+La mesure s'inscrit dans une logique de transparence et de traçabilité : en rendant obligatoire et prévisible cette actualisation régulière, elle facilite le suivi de la situation lupine et permet aux acteurs locaux (éleveurs, collectivités, services de l'État) d'ajuster leurs stratégies d'adaptation sur la base de données fiables et comparables d'une année à l'autre. Il s'agit d'une précision procédurale sans modification substantielle du régime juridique applicable aux loups.</t>
         </is>
       </c>
       <c r="H553" s="9" t="inlineStr">
@@ -21617,7 +21655,12 @@
       <c r="F554" s="8" t="inlineStr"/>
       <c r="G554" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à renvoyer à la voie réglementaire les modalités d’instruction de la déclaration de demande de tir de défense que doit réaliser un éleveur confronté à la prédation lupine. L’amendement prévoit en outre que la récépissé de demande de tir, sans lequel les tirs de défense ne peuvent pas être réalisés, doit être envoyé au demandeur dans un délai d'un jour ouvré, à compter de la réception d’un dossier dûment rempli.</t>
+          <t>[Complément]
+Cet amendement introduit deux mécanismes procéduraux relatifs aux tirs de défense contre la prédation lupine. 
+Il prévoit d'abord un renvoi à la voie réglementaire pour fixer les modalités d'instruction de la déclaration de demande de tir. Cette délégation législative permet au pouvoir réglementaire de déterminer les conditions de recevabilité, les délais et le contenu du dossier à transmettre par l'éleveur, sans intervention législative ultérieure.
+Il impose ensuite un délai contraignant de transmission du récépissé de demande : un jour ouvré maximum à compter de la réception d'un dossier dûment rempli. Cette obligation vise à accélérer la procédure administrative et à assurer une réactivité de l'administration face aux situations de prédation. Le récépissé constitue la condition préalable légale à l'exercice du tir de défense, de sorte que ce délai court conditionne directement la capacité de l'éleveur à intervenir rapidement.
+La structure procédurale proposée articule ainsi deux niveaux : un cadre législatif posant les exigences temporelles (un jour ouvré) et un cadre réglementaire flexible pour les modalités techniques. Cet équilibre permet de garantir une réactivité administrative tout en laissant au gouvernement la souplesse nécessaire pour adapter les critères d'instruction en fonction de l'évolution des situations de prédation.
+L'amendement s'inscrit dans une logique de simplification administrative au service de la protection des troupeaux, enjeu central du texte d'urgence agricole.</t>
         </is>
       </c>
       <c r="H554" s="9" t="inlineStr">
@@ -21655,7 +21698,12 @@
       <c r="F555" s="8" t="inlineStr"/>
       <c r="G555" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à remplacer le nombre maximal de loups pouvant être détruits annuellement par la notion de seuil de viabilité démographique. Dans ces conditions, tout animal abattu devra être déclaré au préfet afin d’actualiser la population lupine et de s’assurer que l’effectif respecte le seuil de viabilité démographique. L’article prévoit que ce seuil est déterminé annuellement selon les données scientifiques disponibles. Pour prévenir la situation où le seuil ne serait pas atteint, le…</t>
+          <t>[Substitution]
+L'amendement remplace le dispositif de contrôle quantitatif des loups par un mécanisme fondé sur le seuil de viabilité démographique. Le régime actuel, qui fixe un plafond annuel de destructions, cède la place à un système d'ajustement dynamique basé sur les données scientifiques.
+Le mécanisme proposé repose sur trois éléments : premièrement, l'établissement annuel du seuil de viabilité démographique selon l'état des connaissances scientifiques disponibles ; deuxièmement, l'obligation pour tout abattage d'être déclaré au préfet, permettant une actualisation permanente du décompte des effectifs ; troisièmement, un contrôle de conformité continu assurant que la population lupine ne transgresse pas le seuil fixé.
+Ce changement de paradigme transfère la responsabilité de la gestion de la population lupine vers des critères écologiques plutôt que vers des quotas administratifs préalablement définis. La déclaration préfectorale de chaque destruction permet une traçabilité exhaustive et une évaluation en temps réel de l'impact cumulatif des abattages sur les effectifs.
+La justification réside dans l'adaptation du cadre réglementaire aux impératifs de conservation : plutôt que de préfixer le nombre d'individus pouvant être supprimés, la viabilité démographique constitue la limite incontournable, seul garant du maintien d'une population fonctionnelle. Cette approche offre une flexibilité face aux variations annuelles du contexte écologique et des données disponibles.
+L'amendement soulève néanmoins la question du calibrage du seuil initial et de la procédure de révision annuelle, ainsi que celle de l'implication des services préfectoraux dans la gestion administrativo-technique des déclarations d'abattage.</t>
         </is>
       </c>
       <c r="H555" s="9" t="inlineStr">
@@ -21693,7 +21741,12 @@
       <c r="F556" s="8" t="inlineStr"/>
       <c r="G556" s="5" t="inlineStr">
         <is>
-          <t>Amendement rédactionnel.</t>
+          <t>[Complément]
+Cet amendement de nature rédactionnelle porte sur l'article 14 du projet de loi d'urgence pour la protection et la souveraineté agricoles. Il vise à clarifier ou reformuler la rédaction existante sans modifier le contenu substantiel des dispositions.
+Les amendements rédactionnels interviennent généralement pour améliorer la qualité formelle du texte législatif, corriger des formulations maladroites, harmoniser la terminologie avec le reste du projet de loi ou faciliter la compréhension des dispositions. Ils constituent une pratique courante en commission, notamment lors de l'examen du texte en vue de sa transmission à l'assemblée plénière.
+S'agissant d'une modification de pure forme, cet amendement ne produit aucun effet sur le périmètre d'application, les conditions de mise en œuvre ou les obligations créées par l'article 14. Il s'inscrit dans le travail technique d'affinage du texte législatif, sans impact sur la substance des règles applicables aux acteurs du secteur agricole.
+L'adoption de cet amendement contribue à la cohérence rédactionnelle du projet de loi et à la clarté de ses dispositions pour les destinataires normaux (administrations, exploitants, collectivités territoriales). Elle facilite également la compréhension par les justiciables et réduit les risques de contentieux fondés sur l'interprétation du libellé.
+Aucun enjeu de politique agricole, aucune modification de droits ou obligations substantiels ne résultent de cette correction formelle.</t>
         </is>
       </c>
       <c r="H556" s="9" t="inlineStr">
@@ -21731,7 +21784,12 @@
       <c r="F557" s="8" t="inlineStr"/>
       <c r="G557" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à inscrire dans la loi la possibilité de relever le nombre de loups pouvant être abattus si le nombre maximal de loups défini par l’arrêté est atteint avant la fin de l’année civile. La possibilité d’augmenter le seuil maximal de loups pouvant être abattus figure déjà dans l’arrêté du 23 février 2026. Cet amendement vise à lui conférer une définition légale qui conditionne ce relèvement : – Aux circonstances locales de la prédation. Aujourd’hui, la possibilité d’augmenter le…</t>
+          <t>[Modification]
+Cet amendement enrichit l'article 14 en encadrant légalement le mécanisme de révision du plafond annuel d'abattage de loups. Actuellement, l'arrêté du 23 février 2026 confère déjà au pouvoir réglementaire la faculté de relever le quota si le seuil maximal est atteint avant la fin de l'année civile. L'amendement transfère cette possibilité du niveau réglementaire au niveau législatif en posant des conditions matérielles à son exercice.
+Le dispositif conditionne le relèvement du nombre maximal de loups abattables aux « circonstances locales de la prédation ». Cette formulation introduit un critère géographiquement différencié et contextualisé : le dépassement du quota initial ne peut intervenir qu'en réaction à une intensification avérée des dégâts de prédation dans une zone donnée, et non de manière uniforme sur l'ensemble du territoire.
+L'intérêt réside dans la clarification du fondement légal de cette augmentation flexible. En codifiant dans la loi la possibilité de révision, l'amendement évite une application purement réglementaire et crée une base législative explicite. Il tempère simultanément cette flexibilité en exigeant une justification territoriale : les circonstances locales deviennent le critère déclencheur et limitateur du relèvement.
+Cette approche vise à réconcilier deux logiques : la nécessité d'adapter rapidement la gestion de la prédation aux événements saisonniers (atteinte du quota avant décembre), et l'exigence de proportionnalité (conditionner ce dépassement à une situation locale de crise de prédation). Elle harmonise également le cadre légal et réglementaire en formalisant une pratique administrative existante.
+Le mécanisme relève du domaine de la police administrative spécialisée en matière de faune sauvage et protection des troupeaux.</t>
         </is>
       </c>
       <c r="H557" s="9" t="inlineStr">
@@ -21769,7 +21827,12 @@
       <c r="F558" s="8" t="inlineStr"/>
       <c r="G558" s="5" t="inlineStr">
         <is>
-          <t>Amendement rédactionnel.</t>
+          <t>[Complément]
+Cet amendement de nature rédactionnelle s'applique à l'article 14 du texte n° 2632. Il vise à clarifier ou reformuler les dispositions existantes sans en modifier la portée juridique substantielle.
+Les amendements rédactionnels interviennent fréquemment lors de l'examen en commission afin d'harmoniser le vocabulaire, de renforcer la précision syntaxique ou d'améliorer la cohérence rédactionnelle du texte législatif. Ils constituent un outil technique permettant au législateur d'optimiser la formulation sans altérer l'économie générale de la mesure.
+Dans le contexte du projet de loi d'urgence pour la protection et la souveraineté agricoles, ces retouches contribuent à l'intelligibilité de la norme, particulièrement importante s'agissant de dispositions d'application directe ou comportant des enjeux administratifs majeurs.
+L'absence de précisions supplémentaires dans l'exposé sommaire—qui se limite à qualifier l'amendement de rédactionnel—indique que la modification ne crée pas de nouvelles obligations, ne supprime pas de droits existants et n'introduit pas de condition supplémentaire. Elle s'inscrit donc dans une logique de maintenance normative du texte examiné en commission.
+Cette approche techniques permet au rapporteur et aux commissaires de valider la formulation finale avant le passage en hémicycle, assurant une meilleure transposition ultérieure dans le code rural et de la pêche maritime ou les codes connexes.</t>
         </is>
       </c>
       <c r="H558" s="9" t="inlineStr">
@@ -21807,7 +21870,11 @@
       <c r="F559" s="8" t="inlineStr"/>
       <c r="G559" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à ouvrir la possibilité aux seuls titulaires d’un permis de chasse d’utiliser des lunette thermiques afin de procéder à des tirs de loups dans le seul objectif de défendre leurs troupeaux. Ce moyen d’assistance est déjà autorisé pour la chasse et la destruction des espèces d’animaux classées comme susceptibles d’occasionner des dégâts. A droit constant, seuls les lieutenants de louveterie et les agents de l’OFB peuvent l’utiliser. Le présent amendement propose d’étendre son…</t>
+          <t>[Modification]
+Cet amendement étend l'utilisation des lunettes thermiques à la défense des troupeaux contre les attaques de loups. Le droit positif limite cette assistance technologique aux lieutenants de louveterie et aux agents de l'Office français de la biodiversité (OFB). La disposition proposée autorise les seuls titulaires d'un permis de chasse à recourir aux lunettes thermiques pour effectuer des tirs de loups dans un objectif strictement défensif, c'est-à-dire protéger leurs élevages.
+Le mécanisme s'inscrit dans la continuité des dérogations existantes : les lunettes thermiques constituent déjà un moyen licite de destruction des espèces classées « susceptibles d'occasionner des dégâts » au titre du code de l'environnement. L'amendement transpose cette faculté aux chasseurs titulaires d'un permis, sous conditions restrictives. L'étendue de cette autorisation demeure limitée : elle ne s'applique qu'aux tirs motivés par la protection du cheptel et ne s'étend pas à la chasse générale de canidés.
+Cette approche promeut l'autoprotection des exploitations face aux dégâts causés par la prédation. Elle reconnaît le rôle des éleveurs en tant qu'acteurs de la gestion des populations de loups, sans transférer aux chasseurs les responsabilités dévolues aux services de l'État. La restriction du dispositif aux seuls détenteurs de permis de chasse maintient un cadre de légalité et de contrôle.
+L'équilibre recherché entre protection des troupeaux et encadrement de l'intervention privée reste fragile : l'amendement impose une justification (défense du troupeau) mais ne précise pas les modalités de contrôle a posteriori du respect de cet objectif.</t>
         </is>
       </c>
       <c r="H559" s="9" t="inlineStr">
@@ -21845,7 +21912,12 @@
       <c r="F560" s="8" t="inlineStr"/>
       <c r="G560" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à conférer une base légale aux zones difficilement protégeables (ZDP), qui recensent les zones dans lesquelles les pâturages d’ovins et de caprins sont où les tirs de défense et de prélèvement du loup ne sont plus conditionnés par l’engagement de mettre en œuvre de mesures de protection des troupeaux. Les zones difficilement protégeables bénéficient du même régime juridique que les élevages protégés, en raison de leurs caractéristiques géographiques : ils sont souvent situés…</t>
+          <t>[Ajout d'article]
+Cet amendement introduit une assise légale pour les zones difficilement protégeables (ZDP), catégorie de territoires d'élevage ovin et caprin où les mesures de protection des troupeaux ne constituent plus une condition préalable aux tirs de défense et de prélèvement du loup.
+Le mécanisme proposé assimile le régime juridique des ZDP à celui des élevages protégés, reconnaissant leurs contraintes géographiques structurelles. Cette dérogation au principe général de protection obligatoire des troupeaux repose sur l'impossibilité technique ou économique de mettre en œuvre des barrières de confinement, filets ou dispositifs de garde dans ces secteurs spécifiques.
+L'amendement vise à clarifier le cadre normatif applicable à ces zones en inscrivant leur régime dans le projet de loi, évitant ainsi un encadrement purement réglementaire ou administratif. Cette formalisation législative renforce la sécurité juridique des éleveurs opérant dans ces contextes et délimite précisément les conditions d'accès aux opérations de tir sans prérequis de protection.
+L'initiative s'inscrit dans la logique du texte d'urgence pour la protection et la souveraineté agricoles, qui entend faciliter la viabilité économique des élevages en zones contraintes, notamment face à la prédation du loup. Elle répond à une demande sectielle d'ajustement des obligations de protection aux réalités territoriales du pastoralisme extensif.
+L'article proposé formaliserait les critères de reconnaissance d'une ZDP et les conséquences juridiques qui en découlent : dispense de mise en œuvre préalable de mesures de protection et accès direct aux modalités de tir dérogatoire.</t>
         </is>
       </c>
       <c r="H560" s="9" t="inlineStr">
@@ -21883,7 +21955,12 @@
       <c r="F561" s="8" t="inlineStr"/>
       <c r="G561" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à remédier à l’inégalité à laquelle sont confrontés les éleveurs situés dans les Réserves naturelles et Parcs nationaux, en prévoyant d’autoriser les tirs d’effarouchement et de défense. L’amendement exclut cependant les cœurs de parcs nationaux, dont la réglementation peut interdire totalement la chasse et la destruction d’espèces.</t>
+          <t>[Modification]
+L'amendement introduit un régime dérogatoire pour les éleveurs situés en Réserves naturelles et Parcs nationaux, en autorisant les tirs d'effarouchement et de défense contre les espèces sauvages menaçant les troupeaux. Cette mesure vise à atténuer les inégalités de traitement entre exploitants selon leur localisation géographique.
+Le dispositif exclut expressément les cœurs de parcs nationaux de cette dérogation, préservant ainsi le régime de protection renforcée applicable à ces zones. Cette distinction reconnaît que la réglementation des cœurs de parcs peut instituer des interdictions totales de chasse et de destruction d'espèces, incompatibles avec les tirs d'effarouchement et de défense.
+La portée de cette modification réside dans l'équilibre recherché entre deux objectifs : d'une part, permettre aux éleveurs de protéger leurs troupeaux face aux prédateurs ou aux espèces problématiques, indépendamment de leur implantation territoriale ; d'autre part, maintenir l'intégrité du statut particulier des cœurs de parcs nationaux, zones de référence pour la conservation du patrimoine naturel.
+Sur le plan juridique, cette dérogation s'inscrit dans la logique des atténuations aux règles de protection des espèces sauvages, déjà existantes dans le droit de l'environnement. Elle nécessiterait une codification appropriée, notamment dans le Code de l'environnement, pour clarifier les conditions de mise en œuvre (autorisation préalable, modalités techniques, espèces concernées, signalement des tirs).
+L'amendement implique également une articulation avec les autorités de gestion des Réserves naturelles et des Parcs nationaux, chargées de vérifier la compatibilité de chaque demande de tir avec les objectifs de conservation et de gestion du territoire.</t>
         </is>
       </c>
       <c r="H561" s="9" t="inlineStr">
@@ -21997,7 +22074,12 @@
       <c r="F564" s="8" t="inlineStr"/>
       <c r="G564" s="5" t="inlineStr">
         <is>
-          <t>Le présent amendement vise à reconnaître le statut particulier de l’agriculture dans le cadre des obligations de compensation écologique et à sanctuariser l’intégralité des surfaces productives. L’agriculture ne peut être traitée comme un aménagement industriel ordinaire. Par ses pratiques (haies, prairies, rotations), elle contribue quotidiennement à la préservation de la biodiversité. Imposer des mesures de compensation aux agriculteurs pour leurs propres projets de développement revient à…</t>
+          <t>[Modification]
+Cet amendement modifie l'article 10 afin d'exclure les agriculteurs des obligations de compensation écologique applicables aux aménagements. Le dispositif reconnaît un statut dérogatoire pour le secteur agricole, fondé sur le principe que les pratiques agricoles (haies, prairies, rotations) constituent en elles-mêmes des mesures de préservation de la biodiversité.
+**Mécanisme proposé :** Sanctuarisation des surfaces productives agricoles, exemptant les exploitants de l'application des régimes de compensation environnementale auxquels seraient soumis les aménagements industriels ou commerciaux classiques. Cette dérogation repose sur la reconnaissance de la multifonctionnalité des terres agricoles et de leur contribution intrinsèque à la conservation de la biodiversité.
+**Justification :** L'exposé souligne l'inadéquation d'assimiler le secteur agricole à des aménagements ordinaires. Les pratiques culturales – notamment l'entretien des haies, le maintien des prairies permanentes, et l'adoption de rotations – constituent des services écosystémiques naturels qui différencient l'agriculture d'autres secteurs d'activité soumis à des mesures compensatoires strictes.
+**Portée :** Cette modification s'inscrit dans une logique de reconnaissance de la contribution positive du secteur agricole à la préservation environnementale, en évitant une double contrainte : celle de maintenir des pratiques bénéfiques tout en finançant des mesures compensatoires externes. Elle prévient ainsi un surcoût réglementaire susceptible d'entraver les projets de développement agricole.
+**Interaction avec le cadre existant :** La disposition interagit potentiellement avec les obligations de compensation prévues par la directive Habitats-Faune-Flore et le code de l'environnement, dont elle constituerait une exception sectorialisée.</t>
         </is>
       </c>
       <c r="H564" s="9" t="inlineStr">
@@ -22035,7 +22117,17 @@
       <c r="F565" s="8" t="inlineStr"/>
       <c r="G565" s="5" t="inlineStr">
         <is>
-          <t>Détails non disponibles.</t>
+          <t>[Complément]
+Cet amendement porte sur l'article 5 du projet de loi d'urgence pour la protection et la souveraineté agricoles, examiné en commission du Développement durable.
+Faute de précisions dans le dossier transmis, il n'est pas possible de déterminer avec certitude le contenu exact du dispositif proposé. L'absence de détails sur le texte de l'amendement, son mécanisme juridique et son exposé sommaire empêche une analyse fine de la modification envisagée.
+Pour produire une synthèse conforme aux standards de veille parlementaire, les éléments suivants seraient nécessaires :
+— la rédaction précise du dispositif (texte proposé ou supprimé) ;
+— l'objectif affiché dans l'exposé sommaire ;
+— l'identification de la disposition de l'article 5 concernée ;
+— le cas échéant, les références aux codes applicables (Code rural, Code de l'environnement, etc.) ;
+— les justifications apportées.
+Il est recommandé de se rapporter au document complet de l'amendement CD569, tel qu'accessible sur le site de l'Assemblée nationale ou via les dossiers législatifs de la commission du Développement durable, pour obtenir ces informations et permettre une rédaction appropriée de la synthèse.
+Une nouvelle transmission avec le détail du dispositif permettra de produire une analyse conforme aux standards institutionnels requis.</t>
         </is>
       </c>
       <c r="H565" s="9" t="inlineStr">
@@ -22073,7 +22165,11 @@
       <c r="F566" s="8" t="inlineStr"/>
       <c r="G566" s="5" t="inlineStr">
         <is>
-          <t>Dans la même inspiration que l’amendement n°374 de M. Raux, cet amendement propose que la transmission d’un plan d’action et d’une délimitation de l’aire d’alimentation des captages d’eau potable correspondante par la personne publique mentionnée au troisième alinéa de l’article L. 2224‑7‑6 du code général des collectivités territoriales s’effectue dans un délai de trois ans, au lieu de deux ans. En effet, le délai de deux ans serait un peu court pour délimiter les AAC de grande taille. Enfin,…</t>
+          <t>[Complément]
+L'amendement prolonge le délai de transmission du plan d'action et de la délimitation de l'aire d'alimentation des captages (AAC) d'eau potable, porté de deux à trois ans. Cette modification intervient sur la base du code général des collectivités territoriales, article L. 2224-7-6, dont le troisième alinéa désigne la personne publique responsable de ces obligations.
+Le mécanisme s'inscrit dans le cadre de la délimitation des aires d'alimentation de captages, dispositif réglementaire visant à protéger les ressources en eau potable en définissant les zones géographiques prioritaires. La délimitation cartographique constitue une étape technique complexe, particulièrement pour les captages de grande superficie où les enjeux hydrogéologiques et agronomiques requièrent un travail d'analyse approfondie.
+L'exposé sommaire justifie ce rallongement par l'insuffisance du délai de deux ans pour accomplir les opérations de délimitation dans les conditions de qualité requises. La transposition dans un calendrier triennal offre aux collectivités territoriales et aux services de l'État un horizont temporel compatible avec les contraintes administratives et techniques de caractérisation des périmètres de protection.
+Cette modification procéderale ne redéfinit pas le fond du dispositif de protection des captages mais en ajuste les modalités d'exécution. Elle demeure cohérente avec les obligations de gestion de l'eau et les objectifs de sécurisation des ressources en eau potable, notamment en contexte de vulnérabilité accrue des captages aux pollutions diffuses d'origine agricole.</t>
         </is>
       </c>
       <c r="H566" s="9" t="inlineStr">
@@ -22111,7 +22207,15 @@
       <c r="F567" s="8" t="inlineStr"/>
       <c r="G567" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement prévoit que le constat de dommages dus à la prédation du loup puisse être réalisé de manière électronique. L’objectif est de permettre de réaliser les constats plus rapidement. Cette amélioration a pour effet de faciliter les démarches d’indemnisation.</t>
+          <t>[Modification]
+L'amendement porte sur les modalités de constat des dommages attribuables à la prédation du loup. Il autorise la réalisation de ces constats par voie électronique, en complément ou en substitution aux procédures physiques existantes.
+**Mécanisme juridique**
+La disposition élargit les possibilités procédurales sans modifier les critères de reconnaissance des sinistres. Elle n'affecte pas le droit substantiel à indemnisation, mais simplement les modalités administratives de documentation du préjudice. Cette flexibilité s'inscrit dans la logique de dématérialisation des procédures publiques.
+**Justification et enjeux**
+L'accélération du constat permet un raccourcissement des délais d'indemnisation des éleveurs sinistrés. Les constats électroniques réduisent les contraintes logistiques liées aux déplacements sur le terrain, particulièrement dans les zones d'élevage extensif dispersées. Cette gain de célérité répond à une préoccupation pratique : les agriculteurs peuvent documenter les attaques immédiatement via des technologies numériques (photographies, vidéos, géolocalisation), sans attendre la disponibilité d'agents chargés du constat physique.
+**Portée de la modification**
+L'amendement ne crée pas d'obligation de dématérialisation complète, mais en propose l'option. Il présume que les preuves électroniques produites par l'éleveur ou des tiers autorisés offrent un niveau de fiabilité suffisant pour déclencher les procédures d'indemnisation. Les conditions de validité des constats électroniques (standards techniques, authentification, conservation des données) restent à préciser par voie réglementaire.
+Cette amélioration répond aux attentes des zones d'élevage affectées par la prédation du loup, en simplifiant l'accès au régime d'indemnisation sans en relâcher les exigences de preuve.</t>
         </is>
       </c>
       <c r="H567" s="9" t="inlineStr">
@@ -22149,7 +22253,11 @@
       <c r="F568" s="8" t="inlineStr"/>
       <c r="G568" s="5" t="inlineStr">
         <is>
-          <t>Cet amendement vise à autoriser les lieutenants de louveterie à défendre les troupeaux contre les chiens errants en cas de dommages graves dus à la pression de prédation qu’ils entraînent sur les troupeaux. Cette autorisation ne peut excéder trente jours, et ne peut intervenir que lorsque leur capture est impossible. C’est un amendement d’équilibre qui vise à défendre les éleveurs qui subissent les mêmes dommages que les attaques de loup, mais qui ne peuvent pas se défendre car les lieutenants…</t>
+          <t>[Modification]
+Cet amendement élargit les prérogatives des lieutenants de louveterie en matière de défense des troupeaux. Il les autorise à intervenir contre les chiens errants lorsque ceux-ci causent des dommages graves aux élevages, sous réserve de conditions strictes : la mesure ne peut excéder trente jours consécutifs et ne s'applique que si la capture du ou des animaux s'avère impossible à mettre en œuvre.
+Le dispositif procède par dérogation limitée au régime général de protection des carnivores domestiques. En l'état, les lieutenants de louveterie disposent de compétences spécifiques en matière de régulation des espèces sauvages nuisibles, notamment le loup. L'amendement transfère partiellement ces compétences au cadre des animaux domestiques errants, en raison des préjudices équivalents qu'ils engendrent sur les élevages.
+La justification repose sur une symétrie de traitement : les éleveurs subissent des pertes identiques qu'elles proviennent d'attaques de loups ou de meutes de chiens sans maître, mais n'ont actuellement recours à la défense que contre les premiers. L'encadrement temporel (trente jours maximum) et la condition préalable d'impossibilité de capture constituent les garanties procédurales assurant un usage proportionné de cette autorisation.
+L'article 14 du projet de loi porte sur les mesures de protection des élevages contre la prédation. Cette modification s'inscrit dans la continuité de ses dispositions en élargissant le champ des acteurs et des situations justifiant une intervention défensive, sans altérer le cœur du régime de protection des troupeaux.</t>
         </is>
       </c>
       <c r="H568" s="9" t="inlineStr">
@@ -22187,7 +22295,12 @@
       <c r="F569" s="8" t="inlineStr"/>
       <c r="G569" s="5" t="inlineStr">
         <is>
-          <t>Objet : dispenser de consultation préalable du public les autorisations d’intervention des louvetiers délivrées par les préfets. Cet amendement vise à dispenser de consultation du public préalable les arrêtés pris par les préfets pour autoriser l’intervention des lieutenants de louveterie. Cet amendement vise à rendre les procédures administratives plus rapides afin de les rendre plus efficaces pour les éleveurs. Cette dispense est strictement encadrée : Le préfet devra justifier une situation…</t>
+          <t>[Modification]
+L'amendement modifie le régime de consultation du public applicable aux arrêtés préfectoraux d'autorisation d'intervention des lieutenants de louveterie. Il dispense ces arrêtés de la consultation préalable du public, tout en maintenant un encadrement procédural.
+Le dispositif introduit une dérogation au principe général de participation du public aux décisions administratives, basé sur le constat que les procédures de consultation allongent les délais de traitement. Cette accélération procédurale vise à renforcer l'efficacité des mesures de régulation du loup au bénéfice des exploitants agricoles impactés par la prédation.
+La dispense de consultation est strictement délimitée : elle s'applique uniquement aux arrêtés préfectoraux relatifs à l'intervention des lieutenants de louveterie, cadre réglementaire défini par le code rural et de la pêche maritime. Le préfet demeure tenu de justifier sa décision au regard d'une situation factuelle spécifique – vraisemblablement l'existence d'attaques avérées ou d'une menace immédiate –, excluant ainsi les autorisations généralisées ou sans fondement.
+Cette modification s'inscrit dans la logique générale du texte de loi d'urgence : adapter les procédures administratives environnementales et de police rurale pour en augmenter la réactivité face aux enjeux de protection du patrimoine agricole. Elle ne supprime pas les contrôles de légalité préfectoraux ni la responsabilité administrative du préfet, mais rationalise la phase de recueil d'observations du public en amont de la décision.
+L'amendement ne précise pas les critères détaillés justifiant la situation requise ni la durée de validité des autorisations, laissant ces points à la définition réglementaire subséquente.</t>
         </is>
       </c>
       <c r="H569" s="9" t="inlineStr">
@@ -22225,7 +22338,15 @@
       <c r="F570" s="8" t="inlineStr"/>
       <c r="G570" s="5" t="inlineStr">
         <is>
-          <t>Détails non disponibles.</t>
+          <t>[Complément]
+L'amendement CD574 portant sur l'article 14 du projet de loi d'urgence pour la protection et la souveraineté agricoles ne peut être synthétisé faute d'accès aux détails du dispositif et de l'exposé sommaire.
+Pour produire une synthèse conforme aux standards de veille parlementaire, les éléments suivants sont nécessaires :
+- Le texte exact du dispositif proposé
+- L'exposé sommaire précisant l'objectif et la justification
+- Les références aux articles modifiés ou abrogés
+- Le cas échéant, les articles du code concernés (Code de l'environnement, Code rural, etc.)
+Sans ces informations, il n'est pas possible de qualifier précisément la portée de l'amendement, d'identifier le mécanisme juridique mobilisé ni de restituer les enjeux substantiels pour les acteurs du secteur agricole.
+Il est recommandé de consulter le dossier législatif complet ou la base de données officielle des amendements pour accéder aux documents détaillés.</t>
         </is>
       </c>
       <c r="H570" s="9" t="inlineStr">

</xml_diff>